<commit_message>
feat: implement Facility, OSRM Routing, and Automatic Cold-Chain Intervention modules
</commit_message>
<xml_diff>
--- a/coldguard_backend/ColdGuard_API_Documentation.xlsx
+++ b/coldguard_backend/ColdGuard_API_Documentation.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="113">
   <si>
     <t>Module</t>
   </si>
@@ -370,6 +370,188 @@
       "confidence_note": "Generated via Gemini AI decision-support model..."
     }
   }
+}</t>
+  </si>
+  <si>
+    <t>Facility</t>
+  </si>
+  <si>
+    <t>/api/facilities</t>
+  </si>
+  <si>
+    <t>List all cold-storage facilities, optionally filtered by status (AVAILABLE/UNAVAILABLE)</t>
+  </si>
+  <si>
+    <t>Query Params:
+status=AVAILABLE</t>
+  </si>
+  <si>
+    <t>{
+  "success": true,
+  "data": [
+    {
+      "id": 1,
+      "name": "ColdGuard Kakkanad Storage B (Demo)",
+      "latitude": 10.0250,
+      "longitude": 76.3500,
+      "capacity": 1500,
+      "available_capacity": 1200,
+      "min_temperature": 2.0,
+      "max_temperature": 8.0,
+      "cost": 650.00,
+      "status": "AVAILABLE"
+    }
+  ]
+}</t>
+  </si>
+  <si>
+    <t>/api/shipments/{id}/facilities/eligible</t>
+  </si>
+  <si>
+    <t>Retrieve eligible cold-storage facilities ranked by approximate distance from truck current GPS</t>
+  </si>
+  <si>
+    <t>{
+  "success": true,
+  "message": "Eligible facilities retrieved and ranked successfully.",
+  "data": {
+    "shipment": { "id": 1, "tracking_number": "CG-2026-VACC-001", "required_temperature": {"min": 2, "max": 8}, "quantity": 500 },
+    "current_location": { "latitude": 10.0159, "longitude": 76.3419 },
+    "facilities": [ {"id": 3, "name": "Aluva Med-Hub Emergency Cold Store", "approximate_distance_km": 1.4, ...} ],
+    "recommended_facility": { "id": 3, "name": "...", "reason": "Eligible temperature range, sufficient capacity..." }
+  }
+}</t>
+  </si>
+  <si>
+    <t>Routing</t>
+  </si>
+  <si>
+    <t>/api/shipments/{id}/location</t>
+  </si>
+  <si>
+    <t>Retrieve latest live truck GPS location and sensor telemetry for continuous tracking</t>
+  </si>
+  <si>
+    <t>{
+  "success": true,
+  "data": {
+    "shipment_id": 1,
+    "tracking_number": "CG-2026-VACC-001",
+    "product_name": "Measles-Rubella (MR) Vaccine",
+    "location": { "latitude": 10.16976, "longitude": 76.24614 },
+    "temperature": 7.8,
+    "humidity": 64.0,
+    "battery": 81.0,
+    "recorded_at": "2026-09-12T12:30:00Z"
+  }
+}</t>
+  </si>
+  <si>
+    <t>/api/shipments/{id}/route</t>
+  </si>
+  <si>
+    <t>Calculate OSRM multi-waypoint road route (Truck -&gt; Facility -&gt; Receiver) with GeoJSON geometry, distance, ETA, and turn-by-turn steps</t>
+  </si>
+  <si>
+    <t>Path Param:
+id=1 or CG-2026-VACC-001
+Query Params:
+facility_id=3</t>
+  </si>
+  <si>
+    <t>{
+  "success": true,
+  "message": "Road route calculated successfully.",
+  "data": {
+    "shipment": { "id": 1, "tracking_number": "CG-2026-VACC-001" },
+    "current_location": { "latitude": 10.16976, "longitude": 76.24614 },
+    "facility": { "id": 3, "name": "Aluva Med-Hub Emergency Cold Store", "latitude": 10.1004, "longitude": 76.3570 },
+    "destination": { "name": "Thrissur District Hospital", "latitude": 10.5276, "longitude": 76.2144 },
+    "distance_km": 78.03,
+    "duration_minutes": 80,
+    "geometry": { "type": "LineString", "coordinates": [[76.24614, 10.16976], ...] },
+    "legs": [...],
+    "steps": [...]
+  }
+}</t>
+  </si>
+  <si>
+    <t>Intervention</t>
+  </si>
+  <si>
+    <t>/api/shipments/{id}/intervention</t>
+  </si>
+  <si>
+    <t>Retrieve current active intervention for a shipment (facility, risk, OSRM route, recipient alerts)</t>
+  </si>
+  <si>
+    <t>{
+  "success": true,
+  "data": {
+    "id": 1,
+    "status": "DIVERTED",
+    "severity": "CRITICAL",
+    "risk_score": 98.0,
+    "reason": "CRITICAL TEMPERATURE BREACH...",
+    "selected_facility": { "id": 3, "name": "Aluva Med-Hub Emergency Cold Store" },
+    "route": { "distance_km": 81.47, "duration_minutes": 82 },
+    "alerts": [...]
+  }
+}</t>
+  </si>
+  <si>
+    <t>/api/shipments/{id}/interventions</t>
+  </si>
+  <si>
+    <t>Retrieve complete historical interventions list for a shipment</t>
+  </si>
+  <si>
+    <t>{
+  "success": true,
+  "data": [ {"id": 1, "status": "RESOLVED", "severity": "CRITICAL", "resolved_at": "ISO-8601", ...} ]
+}</t>
+  </si>
+  <si>
+    <t>/api/shipments/{id}/alerts</t>
+  </si>
+  <si>
+    <t>Retrieve alerts for shipment (supports role filter: MANAGER|DRIVER|RECEIVER)</t>
+  </si>
+  <si>
+    <t>Path Param:
+id=1 or CG-2026-VACC-001
+Query Params:
+role=DRIVER</t>
+  </si>
+  <si>
+    <t>{
+  "success": true,
+  "data": [ {"id": 1, "recipient_role": "DRIVER", "type": "DIVERSION_REQUIRED", "title": "...", "message": "..."} ]
+}</t>
+  </si>
+  <si>
+    <t>/api/interventions/{id}/acknowledge</t>
+  </si>
+  <si>
+    <t>Acknowledge / mark alerts for an intervention as read</t>
+  </si>
+  <si>
+    <t>{
+  "success": true,
+  "message": "Alerts for intervention 1 acknowledged successfully."
+}</t>
+  </si>
+  <si>
+    <t>/api/interventions/{id}/resolve</t>
+  </si>
+  <si>
+    <t>Manually resolve an active intervention</t>
+  </si>
+  <si>
+    <t>{
+  "success": true,
+  "message": "Intervention resolved successfully.",
+  "intervention": { "id": 1, "status": "RESOLVED", "resolved_at": "ISO-8601" }
 }</t>
   </si>
 </sst>
@@ -861,6 +1043,213 @@
         <v>79</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>80</v>
+      </c>
+      <c r="B20" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" t="s">
+        <v>81</v>
+      </c>
+      <c r="D20" t="s">
+        <v>25</v>
+      </c>
+      <c r="E20" t="s">
+        <v>82</v>
+      </c>
+      <c r="F20" t="s">
+        <v>83</v>
+      </c>
+      <c r="G20" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>80</v>
+      </c>
+      <c r="B21" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" t="s">
+        <v>85</v>
+      </c>
+      <c r="D21" t="s">
+        <v>25</v>
+      </c>
+      <c r="E21" t="s">
+        <v>86</v>
+      </c>
+      <c r="F21" t="s">
+        <v>43</v>
+      </c>
+      <c r="G21" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>88</v>
+      </c>
+      <c r="B22" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" t="s">
+        <v>89</v>
+      </c>
+      <c r="D22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E22" t="s">
+        <v>90</v>
+      </c>
+      <c r="F22" t="s">
+        <v>43</v>
+      </c>
+      <c r="G22" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>88</v>
+      </c>
+      <c r="B23" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" t="s">
+        <v>92</v>
+      </c>
+      <c r="D23" t="s">
+        <v>25</v>
+      </c>
+      <c r="E23" t="s">
+        <v>93</v>
+      </c>
+      <c r="F23" t="s">
+        <v>94</v>
+      </c>
+      <c r="G23" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>96</v>
+      </c>
+      <c r="B24" t="s">
+        <v>8</v>
+      </c>
+      <c r="C24" t="s">
+        <v>97</v>
+      </c>
+      <c r="D24" t="s">
+        <v>25</v>
+      </c>
+      <c r="E24" t="s">
+        <v>98</v>
+      </c>
+      <c r="F24" t="s">
+        <v>43</v>
+      </c>
+      <c r="G24" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>96</v>
+      </c>
+      <c r="B25" t="s">
+        <v>8</v>
+      </c>
+      <c r="C25" t="s">
+        <v>100</v>
+      </c>
+      <c r="D25" t="s">
+        <v>25</v>
+      </c>
+      <c r="E25" t="s">
+        <v>101</v>
+      </c>
+      <c r="F25" t="s">
+        <v>43</v>
+      </c>
+      <c r="G25" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>96</v>
+      </c>
+      <c r="B26" t="s">
+        <v>8</v>
+      </c>
+      <c r="C26" t="s">
+        <v>103</v>
+      </c>
+      <c r="D26" t="s">
+        <v>25</v>
+      </c>
+      <c r="E26" t="s">
+        <v>104</v>
+      </c>
+      <c r="F26" t="s">
+        <v>105</v>
+      </c>
+      <c r="G26" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>96</v>
+      </c>
+      <c r="B27" t="s">
+        <v>15</v>
+      </c>
+      <c r="C27" t="s">
+        <v>107</v>
+      </c>
+      <c r="D27" t="s">
+        <v>25</v>
+      </c>
+      <c r="E27" t="s">
+        <v>108</v>
+      </c>
+      <c r="F27" t="s">
+        <v>47</v>
+      </c>
+      <c r="G27" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>96</v>
+      </c>
+      <c r="B28" t="s">
+        <v>15</v>
+      </c>
+      <c r="C28" t="s">
+        <v>110</v>
+      </c>
+      <c r="D28" t="s">
+        <v>25</v>
+      </c>
+      <c r="E28" t="s">
+        <v>111</v>
+      </c>
+      <c r="F28" t="s">
+        <v>47</v>
+      </c>
+      <c r="G28" t="s">
+        <v>112</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>